<commit_message>
Update AAPL data - 2026-09-06 16:10:47
</commit_message>
<xml_diff>
--- a/data/AAPL_data.xlsx
+++ b/data/AAPL_data.xlsx
@@ -4378,7 +4378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:AF2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4499,25 +4499,45 @@
       </c>
       <c r="X1" t="inlineStr">
         <is>
+          <t>book_value</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>price_to_book</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>earnings_growth</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>shares_outstanding</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
           <t>sector</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>industry</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>website</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>last_updated</t>
         </is>
@@ -4553,7 +4573,7 @@
         <v>38272821</v>
       </c>
       <c r="I2" t="n">
-        <v>54390470</v>
+        <v>54154936</v>
       </c>
       <c r="J2" t="n">
         <v>4669700046848</v>
@@ -4601,29 +4621,41 @@
       <c r="W2" t="n">
         <v>1.003</v>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="X2" t="n">
+        <v>7.36</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>43.474186</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>0.287</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>14594180000</v>
+      </c>
+      <c r="AB2" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>Consumer Electronics</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="AD2" t="inlineStr">
         <is>
           <t>https://www.apple.com</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AE2" t="inlineStr">
         <is>
           <t>Apple Inc. designs, manufactures, and markets smartphones, personal computers, tablets, wearables, and accessories worldwide. The company offers iPhone, a line of smartphones; Mac, a line of personal computers; iPad, a line of multi-purpose tablets; and wearables, home, and accessories comprising AirPods, Apple Vision Pro, Apple TV, Apple Watch, Beats products, and HomePod, as well as Apple branded and third-party accessories. It also provides AppleCare support and cloud services; and operates various platforms, including the App Store that allows customers to discover and download applications and digital content, such as books, music, video, games, and podcasts, as well as advertising services include third-party licensing arrangements and its own advertising platforms. In addition, the company offers various subscription-based services, such as Apple Arcade, a game subscription service; Apple Fitness+, a personalized fitness service; Apple Music, which offers users a curated listening experience with on-demand radio stations; Apple News+, a subscription news and magazine service; Apple TV, which offers original content and live sports; Apple Card, a co-branded credit card; and Apple Pay, a cashless payment service, as well as licenses its intellectual property. The company serves consumers, and small and mid-sized businesses; and the education, enterprise, and government markets. It distributes third-party applications for its products through the App Store. The company also sells its products through its retail and online stores, and direct sales force; and third-party cellular network carriers and resellers. The company was formerly known as Apple Computer, Inc. and changed its name to Apple Inc. in January 2007. Apple Inc. was founded in 1976 and is headquartered in Cupertino, California.</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>2026-09-06 05:41:35</t>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>2026-09-06 16:09:38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update AAPL data - 2026-09-06 17:00:22
</commit_message>
<xml_diff>
--- a/data/AAPL_data.xlsx
+++ b/data/AAPL_data.xlsx
@@ -4599,15 +4599,11 @@
       <c r="Q2" t="n">
         <v>0.34</v>
       </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="R2" t="n">
+        <v>0.27618998</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.32623002</v>
       </c>
       <c r="T2" t="n">
         <v>1.4875101</v>
@@ -4655,7 +4651,7 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>2026-09-06 16:48:42</t>
+          <t>2026-09-06 16:59:13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update AAPL data - 2026-09-06 22:21:27
</commit_message>
<xml_diff>
--- a/data/AAPL_data.xlsx
+++ b/data/AAPL_data.xlsx
@@ -4378,7 +4378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF2"/>
+  <dimension ref="A1:AI2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4519,25 +4519,40 @@
       </c>
       <c r="AB1" t="inlineStr">
         <is>
+          <t>total_revenue</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>enterprise_value</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>ebitda</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
           <t>sector</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>industry</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>website</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>last_updated</t>
         </is>
@@ -4629,29 +4644,38 @@
       <c r="AA2" t="n">
         <v>14594180000</v>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AB2" t="n">
+        <v>466822987776</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>4691644645376</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>167959003136</v>
+      </c>
+      <c r="AE2" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AF2" t="inlineStr">
         <is>
           <t>Consumer Electronics</t>
         </is>
       </c>
-      <c r="AD2" t="inlineStr">
+      <c r="AG2" t="inlineStr">
         <is>
           <t>https://www.apple.com</t>
         </is>
       </c>
-      <c r="AE2" t="inlineStr">
+      <c r="AH2" t="inlineStr">
         <is>
           <t>Apple Inc. designs, manufactures, and markets smartphones, personal computers, tablets, wearables, and accessories worldwide. The company offers iPhone, a line of smartphones; Mac, a line of personal computers; iPad, a line of multi-purpose tablets; and wearables, home, and accessories comprising AirPods, Apple Vision Pro, Apple TV, Apple Watch, Beats products, and HomePod, as well as Apple branded and third-party accessories. It also provides AppleCare support and cloud services; and operates various platforms, including the App Store that allows customers to discover and download applications and digital content, such as books, music, video, games, and podcasts, as well as advertising services include third-party licensing arrangements and its own advertising platforms. In addition, the company offers various subscription-based services, such as Apple Arcade, a game subscription service; Apple Fitness+, a personalized fitness service; Apple Music, which offers users a curated listening experience with on-demand radio stations; Apple News+, a subscription news and magazine service; Apple TV, which offers original content and live sports; Apple Card, a co-branded credit card; and Apple Pay, a cashless payment service, as well as licenses its intellectual property. The company serves consumers, and small and mid-sized businesses; and the education, enterprise, and government markets. It distributes third-party applications for its products through the App Store. The company also sells its products through its retail and online stores, and direct sales force; and third-party cellular network carriers and resellers. The company was formerly known as Apple Computer, Inc. and changed its name to Apple Inc. in January 2007. Apple Inc. was founded in 1976 and is headquartered in Cupertino, California.</t>
         </is>
       </c>
-      <c r="AF2" t="inlineStr">
-        <is>
-          <t>2026-09-06 16:59:13</t>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>2026-09-06 22:20:17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update AAPL data - 2026-09-08 08:53:13
</commit_message>
<xml_diff>
--- a/data/AAPL_data.xlsx
+++ b/data/AAPL_data.xlsx
@@ -524,16 +524,16 @@
         <v>45909</v>
       </c>
       <c r="B4" t="n">
-        <v>236.1277593274595</v>
+        <v>236.1277438961264</v>
       </c>
       <c r="C4" t="n">
-        <v>237.901207105354</v>
+        <v>237.9011915581232</v>
       </c>
       <c r="D4" t="n">
-        <v>232.5011563745861</v>
+        <v>232.5011411802574</v>
       </c>
       <c r="E4" t="n">
-        <v>233.4875183105469</v>
+        <v>233.4875030517578</v>
       </c>
       <c r="F4" t="n">
         <v>66313900</v>
@@ -628,16 +628,16 @@
         <v>45915</v>
       </c>
       <c r="B8" t="n">
-        <v>236.1277563565235</v>
+        <v>236.1277410783948</v>
       </c>
       <c r="C8" t="n">
-        <v>237.3133791689625</v>
+        <v>237.3133638141207</v>
       </c>
       <c r="D8" t="n">
-        <v>234.1650054355773</v>
+        <v>234.1649902844441</v>
       </c>
       <c r="E8" t="n">
-        <v>235.828857421875</v>
+        <v>235.8288421630859</v>
       </c>
       <c r="F8" t="n">
         <v>42699500</v>
@@ -680,16 +680,16 @@
         <v>45917</v>
       </c>
       <c r="B10" t="n">
-        <v>238.0905124651219</v>
+        <v>238.09049720761</v>
       </c>
       <c r="C10" t="n">
-        <v>239.216358555688</v>
+        <v>239.2163432260288</v>
       </c>
       <c r="D10" t="n">
-        <v>236.8550706028844</v>
+        <v>236.8550554245431</v>
       </c>
       <c r="E10" t="n">
-        <v>238.1104431152344</v>
+        <v>238.1104278564453</v>
       </c>
       <c r="F10" t="n">
         <v>46508000</v>
@@ -784,16 +784,16 @@
         <v>45923</v>
       </c>
       <c r="B14" t="n">
-        <v>254.9382822522792</v>
+        <v>254.9382669065294</v>
       </c>
       <c r="C14" t="n">
-        <v>256.3929004583055</v>
+        <v>256.3928850249964</v>
       </c>
       <c r="D14" t="n">
-        <v>252.646743968705</v>
+        <v>252.646728760892</v>
       </c>
       <c r="E14" t="n">
-        <v>253.4936065673828</v>
+        <v>253.4935913085938</v>
       </c>
       <c r="F14" t="n">
         <v>60275200</v>
@@ -810,16 +810,16 @@
         <v>45924</v>
       </c>
       <c r="B15" t="n">
-        <v>254.2807025242173</v>
+        <v>254.2806870894418</v>
       </c>
       <c r="C15" t="n">
-        <v>254.7987929994329</v>
+        <v>254.7987775332095</v>
       </c>
       <c r="D15" t="n">
-        <v>250.116078478</v>
+        <v>250.1160632960162</v>
       </c>
       <c r="E15" t="n">
-        <v>251.3814086914062</v>
+        <v>251.3813934326172</v>
       </c>
       <c r="F15" t="n">
         <v>42303700</v>
@@ -836,16 +836,16 @@
         <v>45925</v>
       </c>
       <c r="B16" t="n">
-        <v>252.2781182875964</v>
+        <v>252.2780882048451</v>
       </c>
       <c r="C16" t="n">
-        <v>256.2235509944071</v>
+        <v>256.2235204411851</v>
       </c>
       <c r="D16" t="n">
-        <v>250.7836387354552</v>
+        <v>250.7836088309123</v>
       </c>
       <c r="E16" t="n">
-        <v>255.9246368408203</v>
+        <v>255.9246063232422</v>
       </c>
       <c r="F16" t="n">
         <v>55202100</v>
@@ -888,16 +888,16 @@
         <v>45929</v>
       </c>
       <c r="B18" t="n">
-        <v>253.6231329894407</v>
+        <v>253.6231177228549</v>
       </c>
       <c r="C18" t="n">
-        <v>254.0615160770535</v>
+        <v>254.0615007840798</v>
       </c>
       <c r="D18" t="n">
-        <v>252.0788344590342</v>
+        <v>252.0788192854059</v>
       </c>
       <c r="E18" t="n">
-        <v>253.4936065673828</v>
+        <v>253.4935913085938</v>
       </c>
       <c r="F18" t="n">
         <v>40127700</v>
@@ -940,16 +940,16 @@
         <v>45931</v>
       </c>
       <c r="B20" t="n">
-        <v>254.101347229275</v>
+        <v>254.1013624635733</v>
       </c>
       <c r="C20" t="n">
-        <v>257.8375609779932</v>
+        <v>257.8375764362911</v>
       </c>
       <c r="D20" t="n">
-        <v>253.9917514638179</v>
+        <v>253.9917666915456</v>
       </c>
       <c r="E20" t="n">
-        <v>254.5098419189453</v>
+        <v>254.5098571777344</v>
       </c>
       <c r="F20" t="n">
         <v>48713900</v>
@@ -1018,16 +1018,16 @@
         <v>45936</v>
       </c>
       <c r="B23" t="n">
-        <v>257.0404883747525</v>
+        <v>257.0404730386864</v>
       </c>
       <c r="C23" t="n">
-        <v>258.1165305885388</v>
+        <v>258.1165151882718</v>
       </c>
       <c r="D23" t="n">
-        <v>254.1113214696764</v>
+        <v>254.1113063083761</v>
       </c>
       <c r="E23" t="n">
-        <v>255.7452850341797</v>
+        <v>255.7452697753906</v>
       </c>
       <c r="F23" t="n">
         <v>44664100</v>
@@ -1044,16 +1044,16 @@
         <v>45937</v>
       </c>
       <c r="B24" t="n">
-        <v>255.8648591580886</v>
+        <v>255.8648438796676</v>
       </c>
       <c r="C24" t="n">
-        <v>256.4526841311554</v>
+        <v>256.4526688176338</v>
       </c>
       <c r="D24" t="n">
-        <v>254.4899331102905</v>
+        <v>254.4899179139702</v>
       </c>
       <c r="E24" t="n">
-        <v>255.5360870361328</v>
+        <v>255.5360717773438</v>
       </c>
       <c r="F24" t="n">
         <v>31955800</v>
@@ -1070,16 +1070,16 @@
         <v>45938</v>
       </c>
       <c r="B25" t="n">
-        <v>255.5758888188916</v>
+        <v>255.5759191543519</v>
       </c>
       <c r="C25" t="n">
-        <v>257.5685279874928</v>
+        <v>257.5685585594684</v>
       </c>
       <c r="D25" t="n">
-        <v>255.1673941406971</v>
+        <v>255.1674244276712</v>
       </c>
       <c r="E25" t="n">
-        <v>257.1102294921875</v>
+        <v>257.1102600097656</v>
       </c>
       <c r="F25" t="n">
         <v>36496900</v>
@@ -1096,16 +1096,16 @@
         <v>45939</v>
       </c>
       <c r="B26" t="n">
-        <v>256.8611399345957</v>
+        <v>256.8611554198282</v>
       </c>
       <c r="C26" t="n">
-        <v>257.0504430809132</v>
+        <v>257.0504585775582</v>
       </c>
       <c r="D26" t="n">
-        <v>252.2083294752373</v>
+        <v>252.2083446799687</v>
       </c>
       <c r="E26" t="n">
-        <v>253.1050109863281</v>
+        <v>253.1050262451172</v>
       </c>
       <c r="F26" t="n">
         <v>38322000</v>
@@ -1148,16 +1148,16 @@
         <v>45943</v>
       </c>
       <c r="B28" t="n">
-        <v>248.4621754894735</v>
+        <v>248.462190854235</v>
       </c>
       <c r="C28" t="n">
-        <v>248.7710321191012</v>
+        <v>248.7710475029622</v>
       </c>
       <c r="D28" t="n">
-        <v>244.6562274921306</v>
+        <v>244.6562426215344</v>
       </c>
       <c r="E28" t="n">
-        <v>246.7485046386719</v>
+        <v>246.7485198974609</v>
       </c>
       <c r="F28" t="n">
         <v>38142900</v>
@@ -1252,16 +1252,16 @@
         <v>45947</v>
       </c>
       <c r="B32" t="n">
-        <v>247.1072067041429</v>
+        <v>247.1071917036077</v>
       </c>
       <c r="C32" t="n">
-        <v>252.4474806979352</v>
+        <v>252.447465373221</v>
       </c>
       <c r="D32" t="n">
-        <v>246.3599669580113</v>
+        <v>246.359952002837</v>
       </c>
       <c r="E32" t="n">
-        <v>251.3614807128906</v>
+        <v>251.3614654541016</v>
       </c>
       <c r="F32" t="n">
         <v>49147000</v>
@@ -1278,16 +1278,16 @@
         <v>45950</v>
       </c>
       <c r="B33" t="n">
-        <v>254.9481912125226</v>
+        <v>254.9482209911351</v>
       </c>
       <c r="C33" t="n">
-        <v>263.406949073437</v>
+        <v>263.4069798400544</v>
       </c>
       <c r="D33" t="n">
-        <v>254.6891536205842</v>
+        <v>254.6891833689404</v>
       </c>
       <c r="E33" t="n">
-        <v>261.2748107910156</v>
+        <v>261.2748413085938</v>
       </c>
       <c r="F33" t="n">
         <v>90483000</v>
@@ -1304,16 +1304,16 @@
         <v>45951</v>
       </c>
       <c r="B34" t="n">
-        <v>260.9161783410852</v>
+        <v>260.916147926868</v>
       </c>
       <c r="C34" t="n">
-        <v>264.3136317818121</v>
+        <v>264.313600971564</v>
       </c>
       <c r="D34" t="n">
-        <v>260.8663441185724</v>
+        <v>260.8663137101643</v>
       </c>
       <c r="E34" t="n">
-        <v>261.8028869628906</v>
+        <v>261.8028564453125</v>
       </c>
       <c r="F34" t="n">
         <v>46695900</v>
@@ -1356,16 +1356,16 @@
         <v>45953</v>
       </c>
       <c r="B36" t="n">
-        <v>258.9833552231903</v>
+        <v>258.9832941033833</v>
       </c>
       <c r="C36" t="n">
-        <v>259.6608453480152</v>
+        <v>259.6607840683213</v>
       </c>
       <c r="D36" t="n">
-        <v>257.0604654254083</v>
+        <v>257.0604047594014</v>
       </c>
       <c r="E36" t="n">
-        <v>258.6246643066406</v>
+        <v>258.6246032714844</v>
       </c>
       <c r="F36" t="n">
         <v>32754900</v>
@@ -1382,16 +1382,16 @@
         <v>45954</v>
       </c>
       <c r="B37" t="n">
-        <v>260.2287163700197</v>
+        <v>260.2287466983284</v>
       </c>
       <c r="C37" t="n">
-        <v>263.1578983995789</v>
+        <v>263.1579290692685</v>
       </c>
       <c r="D37" t="n">
-        <v>258.2261042627009</v>
+        <v>258.2261343576155</v>
       </c>
       <c r="E37" t="n">
-        <v>261.8527221679688</v>
+        <v>261.8527526855469</v>
       </c>
       <c r="F37" t="n">
         <v>38253700</v>
@@ -1408,16 +1408,16 @@
         <v>45957</v>
       </c>
       <c r="B38" t="n">
-        <v>263.9051197703755</v>
+        <v>263.9051498417878</v>
       </c>
       <c r="C38" t="n">
-        <v>268.1295048126629</v>
+        <v>268.1295353654346</v>
       </c>
       <c r="D38" t="n">
-        <v>263.6759553344934</v>
+        <v>263.6759853797928</v>
       </c>
       <c r="E38" t="n">
-        <v>267.8206481933594</v>
+        <v>267.8206787109375</v>
       </c>
       <c r="F38" t="n">
         <v>44888200</v>
@@ -1434,16 +1434,16 @@
         <v>45958</v>
       </c>
       <c r="B39" t="n">
-        <v>267.9999758056659</v>
+        <v>268.0000063221084</v>
       </c>
       <c r="C39" t="n">
-        <v>268.896687690681</v>
+        <v>268.8967183092298</v>
       </c>
       <c r="D39" t="n">
-        <v>267.1630710642092</v>
+        <v>267.1631014853557</v>
       </c>
       <c r="E39" t="n">
-        <v>268.0099487304688</v>
+        <v>268.0099792480469</v>
       </c>
       <c r="F39" t="n">
         <v>41534800</v>
@@ -1512,16 +1512,16 @@
         <v>45961</v>
       </c>
       <c r="B42" t="n">
-        <v>275.9705389196515</v>
+        <v>275.9705701844509</v>
       </c>
       <c r="C42" t="n">
-        <v>276.2993413939207</v>
+        <v>276.2993726959702</v>
       </c>
       <c r="D42" t="n">
-        <v>268.1693703205502</v>
+        <v>268.1694007015524</v>
       </c>
       <c r="E42" t="n">
-        <v>269.3749084472656</v>
+        <v>269.3749389648438</v>
       </c>
       <c r="F42" t="n">
         <v>86167100</v>
@@ -1538,16 +1538,16 @@
         <v>45964</v>
       </c>
       <c r="B43" t="n">
-        <v>269.4247673672652</v>
+        <v>269.424736694289</v>
       </c>
       <c r="C43" t="n">
-        <v>269.8531775103368</v>
+        <v>269.8531467885877</v>
       </c>
       <c r="D43" t="n">
-        <v>265.2701011373342</v>
+        <v>265.2700709373508</v>
       </c>
       <c r="E43" t="n">
-        <v>268.0597839355469</v>
+        <v>268.0597534179688</v>
       </c>
       <c r="F43" t="n">
         <v>50194600</v>
@@ -1590,16 +1590,16 @@
         <v>45966</v>
       </c>
       <c r="B45" t="n">
-        <v>267.6213843438783</v>
+        <v>267.6214146886098</v>
       </c>
       <c r="C45" t="n">
-        <v>270.7000385630726</v>
+        <v>270.7000692568828</v>
       </c>
       <c r="D45" t="n">
-        <v>265.9475747682897</v>
+        <v>265.9476049232333</v>
       </c>
       <c r="E45" t="n">
-        <v>269.1457824707031</v>
+        <v>269.1458129882812</v>
       </c>
       <c r="F45" t="n">
         <v>43683100</v>
@@ -1668,16 +1668,16 @@
         <v>45971</v>
       </c>
       <c r="B48" t="n">
-        <v>268.2298525605972</v>
+        <v>268.2298830249396</v>
       </c>
       <c r="C48" t="n">
-        <v>272.9869230403233</v>
+        <v>272.9869540449525</v>
       </c>
       <c r="D48" t="n">
-        <v>266.733924572705</v>
+        <v>266.7339548671466</v>
       </c>
       <c r="E48" t="n">
-        <v>268.6985778808594</v>
+        <v>268.6986083984375</v>
       </c>
       <c r="F48" t="n">
         <v>41312400</v>
@@ -1720,16 +1720,16 @@
         <v>45973</v>
       </c>
       <c r="B50" t="n">
-        <v>274.2535373864602</v>
+        <v>274.253476009827</v>
       </c>
       <c r="C50" t="n">
-        <v>274.9815668240292</v>
+        <v>274.9815052844664</v>
       </c>
       <c r="D50" t="n">
-        <v>270.962507111719</v>
+        <v>270.9624464716027</v>
       </c>
       <c r="E50" t="n">
-        <v>272.7276916503906</v>
+        <v>272.7276306152344</v>
       </c>
       <c r="F50" t="n">
         <v>48398000</v>
@@ -1746,16 +1746,16 @@
         <v>45974</v>
       </c>
       <c r="B51" t="n">
-        <v>273.3658696206449</v>
+        <v>273.3659002679155</v>
       </c>
       <c r="C51" t="n">
-        <v>275.9488654308047</v>
+        <v>275.9488963676571</v>
       </c>
       <c r="D51" t="n">
-        <v>271.3513641926929</v>
+        <v>271.3513946141157</v>
       </c>
       <c r="E51" t="n">
-        <v>272.2090454101562</v>
+        <v>272.2090759277344</v>
       </c>
       <c r="F51" t="n">
         <v>49602800</v>
@@ -1772,16 +1772,16 @@
         <v>45975</v>
       </c>
       <c r="B52" t="n">
-        <v>270.3142081927936</v>
+        <v>270.3141778275755</v>
       </c>
       <c r="C52" t="n">
-        <v>275.2108833889591</v>
+        <v>275.2108524736826</v>
       </c>
       <c r="D52" t="n">
-        <v>268.8681625557137</v>
+        <v>268.8681323529343</v>
       </c>
       <c r="E52" t="n">
-        <v>271.6705322265625</v>
+        <v>271.6705017089844</v>
       </c>
       <c r="F52" t="n">
         <v>47431300</v>
@@ -1824,16 +1824,16 @@
         <v>45979</v>
       </c>
       <c r="B54" t="n">
-        <v>269.25705465795</v>
+        <v>269.2571162750644</v>
       </c>
       <c r="C54" t="n">
-        <v>269.9751013080067</v>
+        <v>269.9751630894399</v>
       </c>
       <c r="D54" t="n">
-        <v>264.5997492422933</v>
+        <v>264.5998097936243</v>
       </c>
       <c r="E54" t="n">
-        <v>266.7139892578125</v>
+        <v>266.7140502929688</v>
       </c>
       <c r="F54" t="n">
         <v>45677300</v>
@@ -1850,16 +1850,16 @@
         <v>45980</v>
       </c>
       <c r="B55" t="n">
-        <v>264.8092197798317</v>
+        <v>264.8091896065648</v>
       </c>
       <c r="C55" t="n">
-        <v>271.4710796703931</v>
+        <v>271.4710487380511</v>
       </c>
       <c r="D55" t="n">
-        <v>264.7793024319747</v>
+        <v>264.7792722621166</v>
       </c>
       <c r="E55" t="n">
-        <v>267.8309936523438</v>
+        <v>267.8309631347656</v>
       </c>
       <c r="F55" t="n">
         <v>40424500</v>
@@ -1954,16 +1954,16 @@
         <v>45986</v>
       </c>
       <c r="B59" t="n">
-        <v>274.5227422872206</v>
+        <v>274.5227726174851</v>
       </c>
       <c r="C59" t="n">
-        <v>279.6188865292943</v>
+        <v>279.6189174225992</v>
       </c>
       <c r="D59" t="n">
-        <v>274.5028075356392</v>
+        <v>274.5028378637012</v>
       </c>
       <c r="E59" t="n">
-        <v>276.2181396484375</v>
+        <v>276.2181701660156</v>
       </c>
       <c r="F59" t="n">
         <v>46914200</v>
@@ -1980,16 +1980,16 @@
         <v>45987</v>
       </c>
       <c r="B60" t="n">
-        <v>276.2082055022192</v>
+        <v>276.2081750495132</v>
       </c>
       <c r="C60" t="n">
-        <v>278.7712367451818</v>
+        <v>278.7712060098946</v>
       </c>
       <c r="D60" t="n">
-        <v>275.8791146523587</v>
+        <v>275.8790842359358</v>
       </c>
       <c r="E60" t="n">
-        <v>276.7966003417969</v>
+        <v>276.7965698242188</v>
       </c>
       <c r="F60" t="n">
         <v>33431400</v>
@@ -2136,16 +2136,16 @@
         <v>45996</v>
       </c>
       <c r="B66" t="n">
-        <v>279.7784559281641</v>
+        <v>279.7784866384076</v>
       </c>
       <c r="C66" t="n">
-        <v>280.3768332578711</v>
+        <v>280.3768640337962</v>
       </c>
       <c r="D66" t="n">
-        <v>277.2951945750906</v>
+        <v>277.2952250127556</v>
       </c>
       <c r="E66" t="n">
-        <v>278.0232238769531</v>
+        <v>278.0232543945312</v>
       </c>
       <c r="F66" t="n">
         <v>47265800</v>
@@ -2214,16 +2214,16 @@
         <v>46001</v>
       </c>
       <c r="B69" t="n">
-        <v>276.9960211276047</v>
+        <v>276.9960515324306</v>
       </c>
       <c r="C69" t="n">
-        <v>278.9905919368044</v>
+        <v>278.9906225605669</v>
       </c>
       <c r="D69" t="n">
-        <v>275.6895796823578</v>
+        <v>275.6896099437804</v>
       </c>
       <c r="E69" t="n">
-        <v>278.0232238769531</v>
+        <v>278.0232543945312</v>
       </c>
       <c r="F69" t="n">
         <v>33038300</v>
@@ -2266,16 +2266,16 @@
         <v>46003</v>
       </c>
       <c r="B71" t="n">
-        <v>277.1455933469186</v>
+        <v>277.1456542987284</v>
       </c>
       <c r="C71" t="n">
-        <v>278.4620173164318</v>
+        <v>278.4620785577587</v>
       </c>
       <c r="D71" t="n">
-        <v>276.068538557602</v>
+        <v>276.0685992725383</v>
       </c>
       <c r="E71" t="n">
-        <v>277.5245666503906</v>
+        <v>277.5246276855469</v>
       </c>
       <c r="F71" t="n">
         <v>39532900</v>
@@ -2500,16 +2500,16 @@
         <v>46017</v>
       </c>
       <c r="B80" t="n">
-        <v>273.4158142002898</v>
+        <v>273.4157529954652</v>
       </c>
       <c r="C80" t="n">
-        <v>274.6225212124231</v>
+        <v>274.6224597374741</v>
       </c>
       <c r="D80" t="n">
-        <v>272.1193247047194</v>
+        <v>272.1192637901173</v>
       </c>
       <c r="E80" t="n">
-        <v>272.6578674316406</v>
+        <v>272.6578063964844</v>
       </c>
       <c r="F80" t="n">
         <v>21521800</v>
@@ -2604,16 +2604,16 @@
         <v>46024</v>
       </c>
       <c r="B84" t="n">
-        <v>271.5209599020358</v>
+        <v>271.5209292436991</v>
       </c>
       <c r="C84" t="n">
-        <v>277.0857995993762</v>
+        <v>277.0857683126949</v>
       </c>
       <c r="D84" t="n">
-        <v>268.2697994337228</v>
+        <v>268.2697691424855</v>
       </c>
       <c r="E84" t="n">
-        <v>270.2743530273438</v>
+        <v>270.2743225097656</v>
       </c>
       <c r="F84" t="n">
         <v>37838100</v>
@@ -2630,16 +2630,16 @@
         <v>46027</v>
       </c>
       <c r="B85" t="n">
-        <v>269.9053759278346</v>
+        <v>269.9053450243044</v>
       </c>
       <c r="C85" t="n">
-        <v>270.7730094869922</v>
+        <v>270.7729784841199</v>
       </c>
       <c r="D85" t="n">
-        <v>265.417590951718</v>
+        <v>265.4175605620285</v>
       </c>
       <c r="E85" t="n">
-        <v>266.5345458984375</v>
+        <v>266.5345153808594</v>
       </c>
       <c r="F85" t="n">
         <v>45647200</v>
@@ -2656,16 +2656,16 @@
         <v>46028</v>
       </c>
       <c r="B86" t="n">
-        <v>266.2752467950493</v>
+        <v>266.275215737747</v>
       </c>
       <c r="C86" t="n">
-        <v>266.8237416838396</v>
+        <v>266.8237105625631</v>
       </c>
       <c r="D86" t="n">
-        <v>261.4084883511094</v>
+        <v>261.4084578614468</v>
       </c>
       <c r="E86" t="n">
-        <v>261.6478271484375</v>
+        <v>261.6477966308594</v>
       </c>
       <c r="F86" t="n">
         <v>52352100</v>
@@ -2682,16 +2682,16 @@
         <v>46029</v>
       </c>
       <c r="B87" t="n">
-        <v>262.485556491205</v>
+        <v>262.4855256371837</v>
       </c>
       <c r="C87" t="n">
-        <v>262.9642340542807</v>
+        <v>262.964203143993</v>
       </c>
       <c r="D87" t="n">
-        <v>259.1047440282917</v>
+        <v>259.1047135716701</v>
       </c>
       <c r="E87" t="n">
-        <v>259.6233215332031</v>
+        <v>259.623291015625</v>
       </c>
       <c r="F87" t="n">
         <v>48309800</v>
@@ -2786,16 +2786,16 @@
         <v>46035</v>
       </c>
       <c r="B91" t="n">
-        <v>258.017707787092</v>
+        <v>258.0176775418968</v>
       </c>
       <c r="C91" t="n">
-        <v>261.0993163539261</v>
+        <v>261.0992857475004</v>
       </c>
       <c r="D91" t="n">
-        <v>257.6886169608135</v>
+        <v>257.6885867541948</v>
       </c>
       <c r="E91" t="n">
-        <v>260.3413696289062</v>
+        <v>260.3413391113281</v>
       </c>
       <c r="F91" t="n">
         <v>45730800</v>
@@ -2812,16 +2812,16 @@
         <v>46036</v>
       </c>
       <c r="B92" t="n">
-        <v>258.7855776250856</v>
+        <v>258.7856080874888</v>
       </c>
       <c r="C92" t="n">
-        <v>261.1092696408236</v>
+        <v>261.1093003767552</v>
       </c>
       <c r="D92" t="n">
-        <v>256.0131254420647</v>
+        <v>256.0131555781144</v>
       </c>
       <c r="E92" t="n">
-        <v>259.2543029785156</v>
+        <v>259.2543334960938</v>
       </c>
       <c r="F92" t="n">
         <v>40019400</v>
@@ -2838,16 +2838,16 @@
         <v>46037</v>
       </c>
       <c r="B93" t="n">
-        <v>259.9424734235133</v>
+        <v>259.9424426175537</v>
       </c>
       <c r="C93" t="n">
-        <v>260.3314293980394</v>
+        <v>260.3313985459844</v>
       </c>
       <c r="D93" t="n">
-        <v>256.352239344094</v>
+        <v>256.3522089636155</v>
       </c>
       <c r="E93" t="n">
-        <v>257.5090942382812</v>
+        <v>257.5090637207031</v>
       </c>
       <c r="F93" t="n">
         <v>39388600</v>
@@ -2864,16 +2864,16 @@
         <v>46038</v>
       </c>
       <c r="B94" t="n">
-        <v>257.1998957308392</v>
+        <v>257.1999111311508</v>
       </c>
       <c r="C94" t="n">
-        <v>258.1971811198186</v>
+        <v>258.1971965798445</v>
       </c>
       <c r="D94" t="n">
-        <v>254.237956908181</v>
+        <v>254.2379721311412</v>
       </c>
       <c r="E94" t="n">
-        <v>254.8363342285156</v>
+        <v>254.8363494873047</v>
       </c>
       <c r="F94" t="n">
         <v>72142800</v>
@@ -2916,16 +2916,16 @@
         <v>46043</v>
       </c>
       <c r="B96" t="n">
-        <v>248.0248902004531</v>
+        <v>248.0249055239374</v>
       </c>
       <c r="C96" t="n">
-        <v>250.8771272171802</v>
+        <v>250.8771427168815</v>
       </c>
       <c r="D96" t="n">
-        <v>244.5144411297041</v>
+        <v>244.5144562363057</v>
       </c>
       <c r="E96" t="n">
-        <v>246.9777374267578</v>
+        <v>246.9777526855469</v>
       </c>
       <c r="F96" t="n">
         <v>54641700</v>
@@ -2968,16 +2968,16 @@
         <v>46045</v>
       </c>
       <c r="B98" t="n">
-        <v>246.6486371992728</v>
+        <v>246.6486524137701</v>
       </c>
       <c r="C98" t="n">
-        <v>248.7329600733879</v>
+        <v>248.7329754164565</v>
       </c>
       <c r="D98" t="n">
-        <v>244.0157890837153</v>
+        <v>244.0158041358057</v>
       </c>
       <c r="E98" t="n">
-        <v>247.3666687011719</v>
+        <v>247.3666839599609</v>
       </c>
       <c r="F98" t="n">
         <v>41689000</v>
@@ -2994,16 +2994,16 @@
         <v>46048</v>
       </c>
       <c r="B99" t="n">
-        <v>250.7973501838168</v>
+        <v>250.7973351598156</v>
       </c>
       <c r="C99" t="n">
-        <v>255.8635622873743</v>
+        <v>255.863546959882</v>
       </c>
       <c r="D99" t="n">
-        <v>249.121917868832</v>
+        <v>249.1219029451975</v>
       </c>
       <c r="E99" t="n">
-        <v>254.7166900634766</v>
+        <v>254.7166748046875</v>
       </c>
       <c r="F99" t="n">
         <v>55969200</v>
@@ -3020,16 +3020,16 @@
         <v>46049</v>
       </c>
       <c r="B100" t="n">
-        <v>258.4664899667647</v>
+        <v>258.4664593428383</v>
       </c>
       <c r="C100" t="n">
-        <v>261.2389423700868</v>
+        <v>261.2389114176715</v>
       </c>
       <c r="D100" t="n">
-        <v>257.5090739976807</v>
+        <v>257.5090434871919</v>
       </c>
       <c r="E100" t="n">
-        <v>257.5689086914062</v>
+        <v>257.5688781738281</v>
       </c>
       <c r="F100" t="n">
         <v>49648300</v>
@@ -3046,16 +3046,16 @@
         <v>46050</v>
       </c>
       <c r="B101" t="n">
-        <v>256.9505880888889</v>
+        <v>256.9506034196754</v>
       </c>
       <c r="C101" t="n">
-        <v>258.1572949521919</v>
+        <v>258.1573103549757</v>
       </c>
       <c r="D101" t="n">
-        <v>253.8191124091609</v>
+        <v>253.8191275531099</v>
       </c>
       <c r="E101" t="n">
-        <v>255.7438812255859</v>
+        <v>255.743896484375</v>
       </c>
       <c r="F101" t="n">
         <v>41288000</v>
@@ -3098,16 +3098,16 @@
         <v>46052</v>
       </c>
       <c r="B103" t="n">
-        <v>254.4773517832236</v>
+        <v>254.4773217725483</v>
       </c>
       <c r="C103" t="n">
-        <v>261.1890792690021</v>
+        <v>261.1890484668085</v>
       </c>
       <c r="D103" t="n">
-        <v>251.4954625126288</v>
+        <v>251.4954328536096</v>
       </c>
       <c r="E103" t="n">
-        <v>258.7756652832031</v>
+        <v>258.775634765625</v>
       </c>
       <c r="F103" t="n">
         <v>92443400</v>
@@ -3124,16 +3124,16 @@
         <v>46055</v>
       </c>
       <c r="B104" t="n">
-        <v>259.3241194003358</v>
+        <v>259.3241487899344</v>
       </c>
       <c r="C104" t="n">
-        <v>269.7557160843994</v>
+        <v>269.7557466562268</v>
       </c>
       <c r="D104" t="n">
-        <v>258.5063380741307</v>
+        <v>258.5063673710488</v>
       </c>
       <c r="E104" t="n">
-        <v>269.2770385742188</v>
+        <v>269.2770690917969</v>
       </c>
       <c r="F104" t="n">
         <v>73913400</v>
@@ -3332,16 +3332,16 @@
         <v>46065</v>
       </c>
       <c r="B112" t="n">
-        <v>275.0990906441111</v>
+        <v>275.0990585104662</v>
       </c>
       <c r="C112" t="n">
-        <v>275.228863950531</v>
+        <v>275.2288318017276</v>
       </c>
       <c r="D112" t="n">
-        <v>259.7165366668213</v>
+        <v>259.7165063299744</v>
       </c>
       <c r="E112" t="n">
-        <v>261.2637939453125</v>
+        <v>261.2637634277344</v>
       </c>
       <c r="F112" t="n">
         <v>81077200</v>
@@ -3592,16 +3592,16 @@
         <v>46080</v>
       </c>
       <c r="B122" t="n">
-        <v>272.3240124520744</v>
+        <v>272.3240439665745</v>
       </c>
       <c r="C122" t="n">
-        <v>272.3240124520744</v>
+        <v>272.3240439665745</v>
       </c>
       <c r="D122" t="n">
-        <v>262.4217010495403</v>
+        <v>262.4217314181026</v>
       </c>
       <c r="E122" t="n">
-        <v>263.7093811035156</v>
+        <v>263.7094116210938</v>
       </c>
       <c r="F122" t="n">
         <v>72366500</v>
@@ -3800,16 +3800,16 @@
         <v>46092</v>
       </c>
       <c r="B130" t="n">
-        <v>260.6248673962081</v>
+        <v>260.624897946549</v>
       </c>
       <c r="C130" t="n">
-        <v>261.6630231774062</v>
+        <v>261.6630538494394</v>
       </c>
       <c r="D130" t="n">
-        <v>259.0876023594815</v>
+        <v>259.0876327296249</v>
       </c>
       <c r="E130" t="n">
-        <v>260.3453674316406</v>
+        <v>260.3453979492188</v>
       </c>
       <c r="F130" t="n">
         <v>26218900</v>
@@ -3826,16 +3826,16 @@
         <v>46093</v>
       </c>
       <c r="B131" t="n">
-        <v>258.1992253881205</v>
+        <v>258.1992408199258</v>
       </c>
       <c r="C131" t="n">
-        <v>258.4887173103141</v>
+        <v>258.4887327594216</v>
       </c>
       <c r="D131" t="n">
-        <v>253.7271951166323</v>
+        <v>253.7272102811576</v>
       </c>
       <c r="E131" t="n">
-        <v>255.3043823242188</v>
+        <v>255.3043975830078</v>
       </c>
       <c r="F131" t="n">
         <v>40794000</v>
@@ -4164,16 +4164,16 @@
         <v>46112</v>
       </c>
       <c r="B144" t="n">
-        <v>247.4683756415328</v>
+        <v>247.4683905467953</v>
       </c>
       <c r="C144" t="n">
-        <v>255.0248824882854</v>
+        <v>255.0248978486836</v>
       </c>
       <c r="D144" t="n">
-        <v>246.6598210163149</v>
+        <v>246.6598358728773</v>
       </c>
       <c r="E144" t="n">
-        <v>253.337890625</v>
+        <v>253.3379058837891</v>
       </c>
       <c r="F144" t="n">
         <v>49598100</v>
@@ -4190,16 +4190,16 @@
         <v>46113</v>
       </c>
       <c r="B145" t="n">
-        <v>253.6273797300248</v>
+        <v>253.6273948962928</v>
       </c>
       <c r="C145" t="n">
-        <v>255.7236296181179</v>
+        <v>255.7236449097363</v>
       </c>
       <c r="D145" t="n">
-        <v>252.8787157917901</v>
+        <v>252.8787309132899</v>
       </c>
       <c r="E145" t="n">
-        <v>255.1746215820312</v>
+        <v>255.1746368408203</v>
       </c>
       <c r="F145" t="n">
         <v>40059400</v>
@@ -4242,16 +4242,16 @@
         <v>46118</v>
       </c>
       <c r="B147" t="n">
-        <v>256.053045051996</v>
+        <v>256.0530752925303</v>
       </c>
       <c r="C147" t="n">
-        <v>261.6929736576745</v>
+        <v>261.6930045642991</v>
       </c>
       <c r="D147" t="n">
-        <v>256.003115847535</v>
+        <v>256.0031460821725</v>
       </c>
       <c r="E147" t="n">
-        <v>258.3988342285156</v>
+        <v>258.3988647460938</v>
       </c>
       <c r="F147" t="n">
         <v>29329900</v>
@@ -4294,16 +4294,16 @@
         <v>46120</v>
       </c>
       <c r="B149" t="n">
-        <v>257.9896016596085</v>
+        <v>257.9896321241455</v>
       </c>
       <c r="C149" t="n">
-        <v>259.2872736156141</v>
+        <v>259.2873042333858</v>
       </c>
       <c r="D149" t="n">
-        <v>256.0730086009651</v>
+        <v>256.0730388391825</v>
       </c>
       <c r="E149" t="n">
-        <v>258.4387817382812</v>
+        <v>258.4388122558594</v>
       </c>
       <c r="F149" t="n">
         <v>41032800</v>
@@ -4320,16 +4320,16 @@
         <v>46121</v>
       </c>
       <c r="B150" t="n">
-        <v>258.5386040524215</v>
+        <v>258.5386343954405</v>
       </c>
       <c r="C150" t="n">
-        <v>260.6548225010532</v>
+        <v>260.6548530924392</v>
       </c>
       <c r="D150" t="n">
-        <v>255.6138310165902</v>
+        <v>255.6138610163474</v>
       </c>
       <c r="E150" t="n">
-        <v>260.0259399414062</v>
+        <v>260.0259704589844</v>
       </c>
       <c r="F150" t="n">
         <v>28121600</v>
@@ -4398,16 +4398,16 @@
         <v>46126</v>
       </c>
       <c r="B153" t="n">
-        <v>258.7881616833942</v>
+        <v>258.7881922504944</v>
       </c>
       <c r="C153" t="n">
-        <v>261.4633801130582</v>
+        <v>261.4634109961452</v>
       </c>
       <c r="D153" t="n">
-        <v>256.7318338868242</v>
+        <v>256.7318642110386</v>
       </c>
       <c r="E153" t="n">
-        <v>258.368896484375</v>
+        <v>258.3689270019531</v>
       </c>
       <c r="F153" t="n">
         <v>48370700</v>
@@ -4450,16 +4450,16 @@
         <v>46128</v>
       </c>
       <c r="B155" t="n">
-        <v>266.3246925362851</v>
+        <v>266.3247234477873</v>
       </c>
       <c r="C155" t="n">
-        <v>266.6840670491935</v>
+        <v>266.6840980024072</v>
       </c>
       <c r="D155" t="n">
-        <v>260.804545264895</v>
+        <v>260.8045755356903</v>
       </c>
       <c r="E155" t="n">
-        <v>262.9307556152344</v>
+        <v>262.9307861328125</v>
       </c>
       <c r="F155" t="n">
         <v>43323100</v>
@@ -4736,16 +4736,16 @@
         <v>46143</v>
       </c>
       <c r="B166" t="n">
-        <v>278.3632116979401</v>
+        <v>278.3632420760759</v>
       </c>
       <c r="C166" t="n">
-        <v>286.7083346607987</v>
+        <v>286.7083659496485</v>
       </c>
       <c r="D166" t="n">
-        <v>277.8740943540899</v>
+        <v>277.8741246788477</v>
       </c>
       <c r="E166" t="n">
-        <v>279.6409606933594</v>
+        <v>279.6409912109375</v>
       </c>
       <c r="F166" t="n">
         <v>79915400</v>
@@ -4762,16 +4762,16 @@
         <v>46146</v>
       </c>
       <c r="B167" t="n">
-        <v>279.1618288412153</v>
+        <v>279.1617980116577</v>
       </c>
       <c r="C167" t="n">
-        <v>280.130102141665</v>
+        <v>280.1300712051751</v>
       </c>
       <c r="D167" t="n">
-        <v>274.3703610857382</v>
+        <v>274.3703307853319</v>
       </c>
       <c r="E167" t="n">
-        <v>276.3368530273438</v>
+        <v>276.3368225097656</v>
       </c>
       <c r="F167" t="n">
         <v>46668400</v>
@@ -4814,16 +4814,16 @@
         <v>46148</v>
       </c>
       <c r="B169" t="n">
-        <v>281.4177950537395</v>
+        <v>281.4178249779708</v>
       </c>
       <c r="C169" t="n">
-        <v>287.5168959460148</v>
+        <v>287.5169265187869</v>
       </c>
       <c r="D169" t="n">
-        <v>280.5693031693742</v>
+        <v>280.5693330033821</v>
       </c>
       <c r="E169" t="n">
-        <v>286.9978332519531</v>
+        <v>286.9978637695312</v>
       </c>
       <c r="F169" t="n">
         <v>58336100</v>
@@ -4840,16 +4840,16 @@
         <v>46149</v>
       </c>
       <c r="B170" t="n">
-        <v>288.7546745760609</v>
+        <v>288.7547052879293</v>
       </c>
       <c r="C170" t="n">
-        <v>291.6095955251437</v>
+        <v>291.6096265406606</v>
       </c>
       <c r="D170" t="n">
-        <v>285.2709015174152</v>
+        <v>285.2709318587503</v>
       </c>
       <c r="E170" t="n">
-        <v>286.9279479980469</v>
+        <v>286.927978515625</v>
       </c>
       <c r="F170" t="n">
         <v>45224300</v>
@@ -10629,7 +10629,7 @@
       </c>
       <c r="AI2" t="inlineStr">
         <is>
-          <t>2026-09-07 03:07:57</t>
+          <t>2026-09-08 08:51:48</t>
         </is>
       </c>
     </row>

</xml_diff>